<commit_message>
Align quality artifacts with day-wise generation
</commit_message>
<xml_diff>
--- a/docs/quality/contenthelper-quality-matrix.xlsx
+++ b/docs/quality/contenthelper-quality-matrix.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6e231a26d65a4f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="2" r:id="Rfc371559738040b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="Re9acf61e65514faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R4ef75950113f4182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Config Dependencies" sheetId="5" r:id="R1d2f2c533e064e85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Evidence" sheetId="6" r:id="R8ac8e1a1f27b4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2543ccdff62e40cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="2" r:id="Re207170a6fe94879"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="R88cd93fc55444a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R685b53a46ba648c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Config Dependencies" sheetId="5" r:id="Rde2ea25fa21b4052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Evidence" sheetId="6" r:id="Rb9f83b1688be44ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -244,9 +244,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -972,16 +972,16 @@
         <x:v>F-009</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Weekly Planning And Generation</x:v>
+        <x:v>Weekly Planning, Daily Generation, And Publish</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>As Manager, I want to plan, generate, review, regenerate, and publish a seven-day content week.</x:v>
+        <x:v>As Manager, I want to generate one day at a time from Daily, accumulate draft cards in the weekly plan container, then review, regenerate, and publish a seven-day week from Weekly.</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Weekly controls handle date windows, brief editing, profile context, idea selection, async AI generation, day review, regeneration, and publish lock.</x:v>
+        <x:v>Daily generates one explicit scheduled date at a time with a non-empty day brief and stores each card in the current weekly_plan draft container. Weekly handles date windows, brief/setup editing, profile context, idea selection, day review, single-day regeneration, and publish lock once seven reviewed cards exist.</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Soft-locked weeks, missing AI key, partial generation, failed day retry, existing published week.</x:v>
+        <x:v>Soft-locked weeks, missing AI key, empty day brief, single-day generation failure, published week lock, date outside selected week.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
         <x:v>TC-028 - TC-046, TC-123 - TC-126, TC-134, TC-178</x:v>
@@ -996,19 +996,19 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>Covered by ManagerAdminUsageTests, GenerateWeekTests, publish-week Deno tests, rendered weekly day-detail UI automation, and final full isolated simulator regression.</x:v>
+        <x:v>Covered by GenerationContractsTests generate_day cases, ManagerAdminUsageTests weekly planning flows, publish-week Deno tests, rendered weekly day-detail UI automation, and hosted E2E day generation.</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="L10" s="9" t="str">
-        <x:v>Generated publish requires complete reviewed seven-card draft.</x:v>
+        <x:v>Publish requires seven reviewed cards in the weekly_plan draft container.</x:v>
       </x:c>
       <x:c r="M10" s="9" t="str">
-        <x:v>WeeklyControlView, AppServices, generate-week, publish-week, write-content.</x:v>
+        <x:v>DayGenerationView, WeeklyControlView, AppServices, generate-week generate_day/regenerate_day, publish-week, write-content.</x:v>
       </x:c>
       <x:c r="N10" s="10" t="str">
-        <x:v>Idea Bank currently selects first open day.</x:v>
+        <x:v>Daily is the generation entry point; Weekly remains review/edit/publish and single-day regeneration.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1272,7 +1272,7 @@
         <x:v>supabase/functions/*, migrations, AppRepositories DTOs.</x:v>
       </x:c>
       <x:c r="N16" s="10" t="str">
-        <x:v>One generate-week partial-progress test was previously ignored.</x:v>
+        <x:v>generate_day and regenerate_day are the supported manager generation actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1371,13 +1371,13 @@
         <x:v>Weekly Setup And Creator Profile Editing</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>As Manager, I want to edit the weekly brief, setup sections, and creator profile before generation so the AI draft reflects current context.</x:v>
+        <x:v>As Manager, I want to edit the weekly brief, setup sections, and creator profile so weekly planning and generation context stay current.</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>The app saves dirty weekly brief/setup/profile edits through write-content before generation-sensitive actions, preserves existing setup sections on failures, and surfaces save errors without replacing current state.</x:v>
+        <x:v>The app saves weekly brief/setup/profile edits through write-content, preserves existing setup sections on failures, and surfaces save errors without replacing current state.</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Dirty brief before generation, save failure, profile update outside weekly setup, missing setup sections.</x:v>
+        <x:v>Weekly brief save failure, profile update outside weekly setup, missing setup sections.</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
         <x:v>TC-139, TC-140, TC-141, TC-174</x:v>
@@ -1404,7 +1404,7 @@
         <x:v>WeeklyControlView, CreatorProfileAdminView, AppServices, write-content.</x:v>
       </x:c>
       <x:c r="N19" s="10" t="str">
-        <x:v>Rendered route coverage verifies field presence and unchanged Saved state; typed edit/save visual QA can expand in the next loop.</x:v>
+        <x:v>Weekly setup context informs day generation but Daily requires its own non-empty day brief.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -1412,16 +1412,16 @@
         <x:v>F-019</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>Weekly Generation Progress And Regeneration</x:v>
+        <x:v>Day Generation And Regeneration</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>As Manager, I want AI generation progress, partial failures, retry, and per-day regeneration to be visible and recoverable.</x:v>
+        <x:v>As Manager, I want single-day generation progress, stable errors, and per-day regeneration to be visible and recoverable.</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Generation emits progress, saves complete drafts, preserves last progress on failure, maps stable error messages, supports one-day regeneration, and protects published/cross-workspace plans.</x:v>
+        <x:v>Daily generate_day emits per-date progress, stores each completed card in the weekly_plan draft container, maps stable error messages, and Weekly regenerate_day updates exactly one draft card while protecting published/cross-workspace plans.</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Missing AI key, invalid generated JSON, stale running days, one failed day, published week lock, date outside selected week.</x:v>
+        <x:v>Missing AI key, empty day brief, invalid generated JSON, one failed day, published week lock, date outside selected week.</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
         <x:v>TC-142, TC-143, TC-144, TC-145</x:v>
@@ -1436,19 +1436,19 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
-        <x:v>Covered by GenerateWeekTests plus Supabase generate-week Deno tests.</x:v>
+        <x:v>Covered by GenerationContractsTests generate_day/regenerate_day cases and Supabase generate-week acceptance plus generate_day/regenerate_day Deno tests.</x:v>
       </x:c>
       <x:c r="K20" s="9" t="str">
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="L20" s="9" t="str">
-        <x:v>Generated draft must contain seven unique scheduled dates for the selected week.</x:v>
+        <x:v>Each generate_day call requires a non-empty day brief and one explicit scheduled date.</x:v>
       </x:c>
       <x:c r="M20" s="9" t="str">
-        <x:v>AppServices, WeeklyGenerationRepository, generate-week Edge Function.</x:v>
+        <x:v>DayGenerationView, WeeklyControlView, AppServices, DayGenerationRepository, generate-week generate_day/regenerate_day.</x:v>
       </x:c>
       <x:c r="N20" s="10" t="str">
-        <x:v>One backend partial-progress scenario remains intentionally ignored.</x:v>
+        <x:v>Cards accumulate in the weekly_plan draft container until seven reviewed cards are ready to publish.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1480,7 +1480,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="J21" s="9" t="str">
-        <x:v>Covered by GenerateWeekTests and publish-week Deno payload tests.</x:v>
+        <x:v>Covered by GenerationContractsTests and publish-week Deno payload tests.</x:v>
       </x:c>
       <x:c r="K21" s="9" t="str">
         <x:v>2026-06-23</x:v>
@@ -1635,13 +1635,13 @@
         <x:v>AI Runway Dashboard</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>As Manager, I want a generation command center that summarizes runtime state, draft state, input context, and idea queue before I generate or regenerate a week.</x:v>
+        <x:v>As Manager, I want a read-only generation dashboard that summarizes runtime state, draft state, input context, and idea queue before I generate from Daily or review from Weekly.</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>AI Runway renders runtime/week/draft/source metrics, latest draft state, input context, and idea queue. Generate/Regenerate triggers current-week generation when AppServices says generation is allowed.</x:v>
+        <x:v>AI Runway renders runtime/week/draft/source metrics, latest draft state, input context, and idea queue. Generation actions live on Daily and Weekly; Runway is read-only.</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>Fixture runtime, no completed generation, generation error, disabled generation while prerequisites are missing.</x:v>
+        <x:v>Fixture runtime, no completed generation, generation error, empty latest draft summary.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
         <x:v>TC-157</x:v>
@@ -1662,13 +1662,13 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="L25" s="9" t="str">
-        <x:v>Generation button requires canGenerateWeek; latest draft block is empty until a generation summary exists.</x:v>
+        <x:v>Latest draft block is empty until day-wise generation has produced a draft summary.</x:v>
       </x:c>
       <x:c r="M25" s="9" t="str">
-        <x:v>AdminShellView, AIRunwayView, AppServices, generate-week.</x:v>
+        <x:v>AdminShellView, AIRunwayView, AppServices, DayGenerationView, WeeklyControlView.</x:v>
       </x:c>
       <x:c r="N25" s="10" t="str">
-        <x:v>Runway is a manager dashboard over the same generation services used by Weekly.</x:v>
+        <x:v>Runway is a manager dashboard over the same day-generation services used by Daily and Weekly.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -2557,13 +2557,13 @@
         <x:v>Generation</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>Generate week</x:v>
+        <x:v>Generate day content from Daily</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>Run generation.</x:v>
+        <x:v>Pick a scheduled date on Daily, enter a non-empty day brief, and run generate_day.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
-        <x:v>Seven-card draft created.</x:v>
+        <x:v>Draft card is created for the target date and stored in the weekly_plan draft container.</x:v>
       </x:c>
       <x:c r="G25" s="9" t="str">
         <x:v>Passed</x:v>
@@ -2573,7 +2573,7 @@
       </x:c>
       <x:c r="I25" s="9" t="str"/>
       <x:c r="J25" s="10" t="str">
-        <x:v>XCTest GenerateWeekTests and hosted E2E generated draft week passed.</x:v>
+        <x:v>XCTest GenerationContractsTests/testGenerateDayCardStoresResultForTheRequestedDate and hosted E2E generate_day passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -2590,10 +2590,10 @@
         <x:v>Publish reviewed week</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>Publish generated draft.</x:v>
+        <x:v>Publish a weekly_plan draft with seven reviewed cards.</x:v>
       </x:c>
       <x:c r="F26" s="9" t="str">
-        <x:v>Creator Today sees card.</x:v>
+        <x:v>Creator Today sees the published card.</x:v>
       </x:c>
       <x:c r="G26" s="9" t="str">
         <x:v>Passed</x:v>
@@ -2603,7 +2603,7 @@
       </x:c>
       <x:c r="I26" s="9" t="str"/>
       <x:c r="J26" s="10" t="str">
-        <x:v>XCTest generated publish and hosted E2E publish/Creator Today checks passed.</x:v>
+        <x:v>XCTest GenerationContractsTests/testPublishingGeneratedDraftPreservesRichFieldsInFixtureModel and hosted E2E publish/Creator Today checks passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -3015,13 +3015,13 @@
         <x:v>Happy path</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>Save dirty weekly brief before generation</x:v>
+        <x:v>Save weekly setup sections</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>Edit weekly brief, start generation.</x:v>
+        <x:v>Edit weekly setup sections and save.</x:v>
       </x:c>
       <x:c r="F40" s="9" t="str">
-        <x:v>Brief save runs before generation and generation continues.</x:v>
+        <x:v>Setup save persists through write-content and the updated sections remain visible.</x:v>
       </x:c>
       <x:c r="G40" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3031,7 +3031,7 @@
       </x:c>
       <x:c r="I40" s="9" t="str"/>
       <x:c r="J40" s="10" t="str">
-        <x:v>XCTest ManagerAdminUsageTests/testGenerateSavesDirtyWeeklyBriefBeforeGenerating; full suite result bundle build-logs/xctest-quality-loop-full-suite-after-publish-fix-20260623.xcresult.</x:v>
+        <x:v>XCTest ManagerAdminUsageTests/testManagerUpdatesWeeklySetupSections.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -3045,13 +3045,13 @@
         <x:v>Error path</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
-        <x:v>Stop generation when weekly brief save fails</x:v>
+        <x:v>Keep weekly setup sections when save fails</x:v>
       </x:c>
       <x:c r="E41" s="9" t="str">
-        <x:v>Make weekly brief save fail, start generation.</x:v>
+        <x:v>Make weekly setup save fail, then retry save.</x:v>
       </x:c>
       <x:c r="F41" s="9" t="str">
-        <x:v>Generation does not proceed and error is stable.</x:v>
+        <x:v>Current setup sections remain unchanged and a stable error is shown.</x:v>
       </x:c>
       <x:c r="G41" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3061,7 +3061,7 @@
       </x:c>
       <x:c r="I41" s="9" t="str"/>
       <x:c r="J41" s="10" t="str">
-        <x:v>XCTest ManagerAdminUsageTests/testGenerateStopsWhenDirtyWeeklyBriefSaveFails.</x:v>
+        <x:v>XCTest ManagerAdminUsageTests/testManagerKeepsWeeklySetupSectionsWhenSaveFails.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
@@ -3091,7 +3091,7 @@
       </x:c>
       <x:c r="I42" s="9" t="str"/>
       <x:c r="J42" s="10" t="str">
-        <x:v>XCTest SupabaseWriteContentDTOTests plus ManagerAdminUsageTests.</x:v>
+        <x:v>XCTest SupabaseWriteContentDTOTests/testUpdateWeeklyBriefRequestEncodesSingleNotesSectionContract plus ManagerAdminUsageTests.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
@@ -3135,13 +3135,13 @@
         <x:v>Happy path</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>Generate complete fixture week</x:v>
+        <x:v>Generate day content with fixture transport</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
-        <x:v>Run fixture generation.</x:v>
+        <x:v>Run fixture generate_day from Daily.</x:v>
       </x:c>
       <x:c r="F44" s="9" t="str">
-        <x:v>Seven-day draft replaces weekly plan and reaches ready-for-review.</x:v>
+        <x:v>Generated draft card is stored for the requested date in the weekly_plan draft container.</x:v>
       </x:c>
       <x:c r="G44" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3151,7 +3151,7 @@
       </x:c>
       <x:c r="I44" s="9" t="str"/>
       <x:c r="J44" s="10" t="str">
-        <x:v>XCTest GenerateWeekTests/testAppServicesGenerationSuccessWithFixtureRepository.</x:v>
+        <x:v>XCTest GenerationContractsTests/testGenerateDayCardStoresResultForTheRequestedDate.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
@@ -3165,13 +3165,13 @@
         <x:v>Error path</x:v>
       </x:c>
       <x:c r="D45" s="9" t="str">
-        <x:v>Surface generation failure without losing progress</x:v>
+        <x:v>Surface single-day generation failures with stable errors</x:v>
       </x:c>
       <x:c r="E45" s="9" t="str">
-        <x:v>Simulate wrapped/stable generation failures.</x:v>
+        <x:v>Reject empty brief, past dates, and wrapped/stable generation failures.</x:v>
       </x:c>
       <x:c r="F45" s="9" t="str">
-        <x:v>Stable message shown and last progress count preserved.</x:v>
+        <x:v>Stable per-date error is shown and other accumulated draft cards remain intact.</x:v>
       </x:c>
       <x:c r="G45" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3181,7 +3181,7 @@
       </x:c>
       <x:c r="I45" s="9" t="str"/>
       <x:c r="J45" s="10" t="str">
-        <x:v>XCTest GenerateWeekTests generation failure cases.</x:v>
+        <x:v>XCTest GenerationContractsTests/testGenerateDayCardRequiresBrief, testGenerateDayCardRejectsPastDates, and generation retry-policy cases.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
@@ -3195,13 +3195,13 @@
         <x:v>Boundary</x:v>
       </x:c>
       <x:c r="D46" s="9" t="str">
-        <x:v>Regenerate one day</x:v>
+        <x:v>Regenerate one day from Weekly</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
         <x:v>Call regenerate_day for one scheduled date.</x:v>
       </x:c>
       <x:c r="F46" s="9" t="str">
-        <x:v>Exactly one draft card changes and other six remain.</x:v>
+        <x:v>Exactly one draft card changes and the other six remain.</x:v>
       </x:c>
       <x:c r="G46" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3211,7 +3211,7 @@
       </x:c>
       <x:c r="I46" s="9" t="str"/>
       <x:c r="J46" s="10" t="str">
-        <x:v>Deno generate-week regenerate_day tests.</x:v>
+        <x:v>Deno generate-week regenerate_day tests and supabase/functions/generate-week/acceptance.ts regenerate_day coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
@@ -3225,7 +3225,7 @@
         <x:v>Permission/security</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
-        <x:v>Reject invalid generation scopes</x:v>
+        <x:v>Reject invalid generate_day and regenerate_day scopes</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
         <x:v>Try creator role, cross-workspace plan, published lock, or date outside week.</x:v>
@@ -3241,7 +3241,7 @@
       </x:c>
       <x:c r="I47" s="9" t="str"/>
       <x:c r="J47" s="10" t="str">
-        <x:v>Deno generate-week index tests; 79 passed, 1 ignored overall.</x:v>
+        <x:v>Deno generate_day/regenerate_day index tests and acceptance.ts creator-role and published-lock checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -3258,7 +3258,7 @@
         <x:v>Publish preserves edited generated rich fields</x:v>
       </x:c>
       <x:c r="E48" s="9" t="str">
-        <x:v>Edit generated caption/backup story then publish.</x:v>
+        <x:v>Edit generated caption/backup story then publish seven reviewed cards.</x:v>
       </x:c>
       <x:c r="F48" s="9" t="str">
         <x:v>Published week cards retain edited rich fields.</x:v>
@@ -3271,7 +3271,7 @@
       </x:c>
       <x:c r="I48" s="9" t="str"/>
       <x:c r="J48" s="10" t="str">
-        <x:v>XCTest GenerateWeekTests/testPublishingGeneratedDraftPreservesRichFieldsInFixtureModel.</x:v>
+        <x:v>XCTest GenerationContractsTests/testPublishingGeneratedDraftPreservesRichFieldsInFixtureModel.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -3395,7 +3395,7 @@
       </x:c>
       <x:c r="I52" s="9" t="str"/>
       <x:c r="J52" s="10" t="str">
-        <x:v>XcodeBuildMCP full regression passed 83/0/0; result bundle /Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-17-44-417Z_pid53980_67490e43.xcresult.</x:v>
+        <x:v>XcodeBuildMCP full regression passed 83/0/0; result bundle &lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-17-44-417Z_pid53980_67490e43.xcresult.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
@@ -3595,7 +3595,7 @@
         <x:v>Launch fixture admin shell and tap Runway.</x:v>
       </x:c>
       <x:c r="F59" s="9" t="str">
-        <x:v>AI Runway dashboard renders runtime, draft, source, latest draft, and input context signals.</x:v>
+        <x:v>AI Runway dashboard renders runtime, draft, source, latest draft, and input context signals without exposing generation actions.</x:v>
       </x:c>
       <x:c r="G59" s="9" t="str">
         <x:v>Passed</x:v>
@@ -3748,7 +3748,7 @@
         <x:v>Live smoke script type check</x:v>
       </x:c>
       <x:c r="E64" s="9" t="str">
-        <x:v>Run deno check against live-write-boundary, live-weekly-setup, ai-weekly-generation, and live-e2e QA scripts.</x:v>
+        <x:v>Run deno check against live-write-boundary, live-weekly-setup, and live-e2e QA scripts.</x:v>
       </x:c>
       <x:c r="F64" s="9" t="str">
         <x:v>All smoke scripts type-check without executing live network mutations.</x:v>
@@ -3761,7 +3761,7 @@
       </x:c>
       <x:c r="I64" s="9" t="str"/>
       <x:c r="J64" s="10" t="str">
-        <x:v>deno check passed for scripts/live-write-boundary-smoke.ts, scripts/live-weekly-setup-smoke.ts, scripts/ai-weekly-generation-smoke.ts, and scripts/qa/live-e2e-qa.ts.</x:v>
+        <x:v>deno check passed for scripts/live-write-boundary-smoke.ts, scripts/live-weekly-setup-smoke.ts, and scripts/qa/live-e2e-qa.ts.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
@@ -4709,7 +4709,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I6" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T05-53-13-948Z_pid92382_78c140a6.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T05-53-13-948Z_pid92382_78c140a6.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -4738,7 +4738,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
-        <x:v>One generate-week partial-progress test is intentionally ignored.</x:v>
+        <x:v>Coverage includes generate_day/regenerate_day contracts via generate-week function tests and acceptance.ts.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -4999,7 +4999,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I16" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-10-13-555Z_pid53980_18de580c.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-10-13-555Z_pid53980_18de580c.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -5028,7 +5028,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I17" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-25-20-849Z_pid53980_18026ff6.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-25-20-849Z_pid53980_18026ff6.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -5086,7 +5086,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I19" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-53-03-762Z_pid53980_a05ad2f9.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-53-03-762Z_pid53980_a05ad2f9.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -5173,7 +5173,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I22" s="10" t="str">
-        <x:v>Release build settings report CURRENT_PROJECT_VERSION=11, MARKETING_VERSION=1.0, PRODUCT_BUNDLE_IDENTIFIER=com.prateekranka.creatorcontenthelper.</x:v>
+        <x:v>Release build settings report CURRENT_PROJECT_VERSION=11, MARKETING_VERSION=1.0, and the expected release bundle identifier.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -5231,7 +5231,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I24" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-27-56-275Z_pid53980_89b99e45.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-27-56-275Z_pid53980_89b99e45.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -5260,7 +5260,7 @@
         <x:v>2026-06-23</x:v>
       </x:c>
       <x:c r="I25" s="10" t="str">
-        <x:v>/Users/prateekranka/Library/Developer/XcodeBuildMCP/workspaces/contenthelper-ui-audit-245d4d5361a6/result-bundles/test_sim_2026-06-23T03-30-21-720Z_pid53980_d5bda32a.xcresult; no warnings.</x:v>
+        <x:v>&lt;XcodeBuildMCP workspace&gt;/result-bundles/test_sim_2026-06-23T03-30-21-720Z_pid53980_d5bda32a.xcresult; no warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">

</xml_diff>